<commit_message>
Fix grouped sources ordering and add RGPH priority + import/export scripts
</commit_message>
<xml_diff>
--- a/Donnees/Statistiques Démographiques et sociales/Education/Taux Net de Scolarisation 2006-2023.xlsx
+++ b/Donnees/Statistiques Démographiques et sociales/Education/Taux Net de Scolarisation 2006-2023.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\Ansade_Project\Donnees\Statistiques Démographiques et sociales\Education\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{629B80E4-447C-40EE-9513-807C541E49AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16A9361C-30DD-40BB-83EE-9DFA71B06E54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Garçons" sheetId="4" r:id="rId1"/>

</xml_diff>